<commit_message>
edit excel file test envi
</commit_message>
<xml_diff>
--- a/Lab4_BVT.xlsx
+++ b/Lab4_BVT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chitsuthasoomlek/Work/Class/SQA/2026/Lab/Lab4_BVT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\Year_3_1\SQA\Lab\Lab4\Lab4_BVT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C045E2D1-995E-144A-A36D-6DBCBA38CDBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B302788-38C4-4B53-95F7-7B7D59F4938E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="29400" windowHeight="17140" activeTab="2" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
+    <workbookView xWindow="9825" yWindow="0" windowWidth="18120" windowHeight="15585" activeTab="2" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="4" r:id="rId1"/>
@@ -23,22 +23,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="93">
   <si>
     <t>Test Case Design and Test Results</t>
   </si>
@@ -236,13 +226,96 @@
   </si>
   <si>
     <t>HRR</t>
+  </si>
+  <si>
+    <t>invalid</t>
+  </si>
+  <si>
+    <t>หมายเหตุ</t>
+  </si>
+  <si>
+    <t>มีแค่ค่า Nom</t>
+  </si>
+  <si>
+    <t>เปลี่ยนค่า VO2 Max</t>
+  </si>
+  <si>
+    <t>เปลี่ยนค่า RHR</t>
+  </si>
+  <si>
+    <t>เปลี่ยนค่า HRR</t>
+  </si>
+  <si>
+    <t>673380286-0</t>
+  </si>
+  <si>
+    <t>พิไลพร คำเวียง</t>
+  </si>
+  <si>
+    <t>totalScore=9,fitnessLevel=STANDARD</t>
+  </si>
+  <si>
+    <t>totalScore=6,fitnessLevel=STANDARD</t>
+  </si>
+  <si>
+    <t>totalScore=11,fitnessLevel=STANDARD</t>
+  </si>
+  <si>
+    <t>totalScore=7,fitnessLevel=STANDARD</t>
+  </si>
+  <si>
+    <t>Throws IllegalArgumentException: "VO2 Max cannot be negative."</t>
+  </si>
+  <si>
+    <t>totalScore=6, fitnessLevel=STANDARD</t>
+  </si>
+  <si>
+    <t>totalScore=11, fitnessLevel=STANDARD</t>
+  </si>
+  <si>
+    <t>Throws IllegalArgumentException: "Resting Heart Rate (RHR) must be between 40 and 220 bpm."</t>
+  </si>
+  <si>
+    <t>totalScore=7, fitnessLevel=STANDARD</t>
+  </si>
+  <si>
+    <t>Throws IllegalArgumentException: "Heart Rate Recovery (HRR) cannot be negative."</t>
+  </si>
+  <si>
+    <t>OS:Windows_NT x64 10.0.26200 / IDE:vs code Version: 1.129.1 (user setup) / JDK:openjdk version "25.0.3" 2026-04-21 LTS</t>
+  </si>
+  <si>
+    <t>df-001</t>
+  </si>
+  <si>
+    <t>ไม่มีขอบบนของ Vo2 max กับ HRR</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>minor</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> validateInputs() 
+เช็คขอบล่างของ VO2 Max (&lt; 0) 
+และ HRR (&lt; 0) แต่ไม่มีการเช็คขอบบน</t>
+  </si>
+  <si>
+    <t>DF-001 (TC007, TC019)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -297,13 +370,21 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="18"/>
-      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="222"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="TH SarabunPSK"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -340,8 +421,43 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -425,14 +541,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -456,12 +597,6 @@
     <xf numFmtId="14" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -474,19 +609,50 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -496,15 +662,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -517,20 +674,49 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 3 4" xfId="1" xr:uid="{DD4AD2A2-321B-5F4E-AAE1-B5C53296010C}"/>
     <cellStyle name="Normal_ftest" xfId="2" xr:uid="{2E60872E-C109-5D40-AEB9-649A4B5FF349}"/>
+    <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
+    <cellStyle name="แย่" xfId="4" builtinId="27"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -863,79 +1049,111 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5CE7BA3-0BEF-0C45-955A-B350FDBEC636}">
   <dimension ref="A2:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="27" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="27" x14ac:dyDescent="0.6"/>
   <cols>
-    <col min="1" max="1" width="33.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="17.1640625" style="1" customWidth="1"/>
-    <col min="3" max="6" width="9.1640625" style="1"/>
-    <col min="7" max="7" width="21.83203125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.1640625" style="1"/>
+    <col min="1" max="1" width="33.875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.125" style="1" customWidth="1"/>
+    <col min="3" max="6" width="9.125" style="1"/>
+    <col min="7" max="7" width="21.875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="56" x14ac:dyDescent="0.45">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:7" ht="54" x14ac:dyDescent="0.6">
+      <c r="A2" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="14" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="17"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B3" s="51">
+        <v>13</v>
+      </c>
+      <c r="C3" s="51">
+        <v>13</v>
+      </c>
+      <c r="D3" s="51">
+        <v>0</v>
+      </c>
+      <c r="E3" s="51">
+        <v>0</v>
+      </c>
+      <c r="F3" s="51">
+        <v>0</v>
+      </c>
+      <c r="G3" s="52"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B4" s="51">
+        <v>19</v>
+      </c>
+      <c r="C4" s="51">
+        <v>19</v>
+      </c>
+      <c r="D4" s="51">
+        <v>0</v>
+      </c>
+      <c r="E4" s="51">
+        <v>0</v>
+      </c>
+      <c r="F4" s="51">
+        <v>0</v>
+      </c>
+      <c r="G4" s="51" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A6" s="21" t="s">
+      <c r="B5" s="51"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.6">
+      <c r="A6" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="20"/>
+      <c r="B6" s="51">
+        <v>32</v>
+      </c>
+      <c r="C6" s="53">
+        <v>32</v>
+      </c>
+      <c r="D6" s="54">
+        <v>0</v>
+      </c>
+      <c r="E6" s="51">
+        <v>0</v>
+      </c>
+      <c r="F6" s="51">
+        <v>0</v>
+      </c>
+      <c r="G6" s="55"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -944,831 +1162,1392 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFEE3D1E-0814-D34A-9C7B-86FDE5AD12C8}">
-  <dimension ref="A1:M28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="27" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:N28"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="27" x14ac:dyDescent="0.6"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" style="1" customWidth="1"/>
-    <col min="2" max="4" width="21.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.1640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="25.1640625" style="1" customWidth="1"/>
-    <col min="8" max="10" width="10.83203125" style="1"/>
-    <col min="11" max="11" width="15.33203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" style="1"/>
-    <col min="13" max="13" width="16.5" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="17.625" style="1" customWidth="1"/>
+    <col min="2" max="4" width="21.375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="35.625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="38.375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="25.125" style="1" customWidth="1"/>
+    <col min="9" max="11" width="10.875" style="1"/>
+    <col min="12" max="12" width="15.375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="10.875" style="1"/>
+    <col min="14" max="14" width="16.5" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="26"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="8" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="35"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="N1" s="8" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="G2" s="4"/>
-      <c r="J2" s="3" t="s">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="H2" s="4"/>
+      <c r="K2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="L2" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="N2" s="22" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="6"/>
-      <c r="J3" s="3" t="s">
+      <c r="G3" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="H3" s="30"/>
+      <c r="K3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="L3" s="6">
+        <v>0</v>
+      </c>
+      <c r="M3" s="6">
+        <v>40</v>
+      </c>
+      <c r="N3" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="J4" s="3" t="s">
+      <c r="G4" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" s="30"/>
+      <c r="K4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="L4" s="6">
+        <v>1</v>
+      </c>
+      <c r="M4" s="6">
+        <v>41</v>
+      </c>
+      <c r="N4" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
+      <c r="B5" s="46" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="45"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="6"/>
-      <c r="J5" s="3" t="s">
+      <c r="G5" s="31">
+        <v>244548</v>
+      </c>
+      <c r="H5" s="32"/>
+      <c r="K5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J6" s="3" t="s">
+      <c r="L5" s="6">
+        <v>45</v>
+      </c>
+      <c r="M5" s="6">
+        <v>72</v>
+      </c>
+      <c r="N5" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="K6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-    </row>
-    <row r="7" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="33" t="s">
+      <c r="L6" s="6">
+        <v>99</v>
+      </c>
+      <c r="M6" s="6">
+        <v>219</v>
+      </c>
+      <c r="N6" s="6">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A7" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="33" t="s">
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="33" t="s">
+      <c r="F7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="34" t="s">
+      <c r="G7" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="H7" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A8" s="33"/>
-      <c r="B8" s="8" t="s">
+      <c r="L7" s="6">
+        <v>100</v>
+      </c>
+      <c r="M7" s="6">
+        <v>220</v>
+      </c>
+      <c r="N7" s="6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A8" s="39"/>
+      <c r="B8" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="34"/>
-      <c r="J8" s="3" t="s">
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="41"/>
+      <c r="K8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="L8" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="N8" s="22" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B9" s="17">
+        <v>45</v>
+      </c>
+      <c r="C9" s="17">
+        <v>72</v>
+      </c>
+      <c r="D9" s="17">
+        <v>15</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B10" s="18">
+        <v>0</v>
+      </c>
+      <c r="C10" s="43">
+        <v>72</v>
+      </c>
+      <c r="D10" s="43">
+        <v>15</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" s="26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="J11" s="2"/>
+      <c r="B11" s="18">
+        <v>1</v>
+      </c>
+      <c r="C11" s="43">
+        <v>72</v>
+      </c>
+      <c r="D11" s="43">
+        <v>15</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="27"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A12" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="J12" s="2"/>
+      <c r="B12" s="18">
+        <v>99</v>
+      </c>
+      <c r="C12" s="43">
+        <v>72</v>
+      </c>
+      <c r="D12" s="43">
+        <v>15</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" s="27"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A13" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="J13" s="2"/>
+      <c r="B13" s="18">
+        <v>100</v>
+      </c>
+      <c r="C13" s="43">
+        <v>72</v>
+      </c>
+      <c r="D13" s="43">
+        <v>15</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" s="28"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N13" s="2"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A14" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="J14" s="2"/>
+      <c r="B14" s="43">
+        <v>45</v>
+      </c>
+      <c r="C14" s="19">
+        <v>40</v>
+      </c>
+      <c r="D14" s="43">
+        <v>15</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="26" t="s">
+        <v>70</v>
+      </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A15" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="J15" s="2"/>
+      <c r="B15" s="43">
+        <v>45</v>
+      </c>
+      <c r="C15" s="19">
+        <v>41</v>
+      </c>
+      <c r="D15" s="43">
+        <v>15</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="27"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N15" s="2"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A16" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="J16" s="2"/>
+      <c r="B16" s="43">
+        <v>45</v>
+      </c>
+      <c r="C16" s="19">
+        <v>219</v>
+      </c>
+      <c r="D16" s="43">
+        <v>15</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="27"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A17" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="J17" s="2"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B17" s="43">
+        <v>45</v>
+      </c>
+      <c r="C17" s="19">
+        <v>220</v>
+      </c>
+      <c r="D17" s="43">
+        <v>15</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" s="28"/>
+      <c r="K17" s="2"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="J18" s="2"/>
+      <c r="B18" s="43">
+        <v>45</v>
+      </c>
+      <c r="C18" s="43">
+        <v>72</v>
+      </c>
+      <c r="D18" s="24">
+        <v>0</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H18" s="26" t="s">
+        <v>71</v>
+      </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N18" s="2"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A19" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B19" s="43">
+        <v>45</v>
+      </c>
+      <c r="C19" s="43">
+        <v>72</v>
+      </c>
+      <c r="D19" s="24">
+        <v>1</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H19" s="27"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A20" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B20" s="43">
+        <v>45</v>
+      </c>
+      <c r="C20" s="43">
+        <v>72</v>
+      </c>
+      <c r="D20" s="24">
+        <v>29</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H20" s="27"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A21" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="J21" s="2"/>
+      <c r="B21" s="43">
+        <v>45</v>
+      </c>
+      <c r="C21" s="43">
+        <v>72</v>
+      </c>
+      <c r="D21" s="24">
+        <v>30</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H21" s="28"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J22" s="2"/>
+      <c r="N21" s="2"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.6">
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J23" s="2"/>
+      <c r="N22" s="2"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.6">
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J24" s="2"/>
+      <c r="N23" s="2"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.6">
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J25" s="2"/>
+      <c r="N24" s="2"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.6">
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J26" s="2"/>
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.6">
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J27" s="2"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J28" s="2"/>
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="K27" s="2"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.6">
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="16">
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F7:F8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="A7:A8"/>
     <mergeCell ref="G7:G8"/>
-    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3A52C6A-99BA-484C-B915-27B6FC4D32AF}">
-  <dimension ref="A1:M28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="27" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:N28"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="27" x14ac:dyDescent="0.6"/>
   <cols>
-    <col min="1" max="1" width="19.83203125" style="1" customWidth="1"/>
-    <col min="2" max="4" width="21.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.1640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="25.1640625" style="1" customWidth="1"/>
-    <col min="8" max="10" width="10.83203125" style="1"/>
-    <col min="11" max="11" width="15.33203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" style="1"/>
-    <col min="13" max="13" width="16.5" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="19.875" style="1" customWidth="1"/>
+    <col min="2" max="4" width="21.375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="89.875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="51.875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="25.125" style="1" customWidth="1"/>
+    <col min="9" max="11" width="10.875" style="1"/>
+    <col min="12" max="12" width="15.375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="10.875" style="1"/>
+    <col min="14" max="14" width="16.5" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="26"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="8" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="35"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="N1" s="8" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="G2" s="4"/>
-      <c r="J2" s="3" t="s">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="H2" s="4"/>
+      <c r="K2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="L2" s="6">
+        <v>-1</v>
+      </c>
+      <c r="M2" s="6">
+        <v>39</v>
+      </c>
+      <c r="N2" s="6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="6"/>
-      <c r="J3" s="3" t="s">
+      <c r="G3" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="H3" s="30"/>
+      <c r="K3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="L3" s="6">
+        <v>0</v>
+      </c>
+      <c r="M3" s="6">
+        <v>40</v>
+      </c>
+      <c r="N3" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="J4" s="3" t="s">
+      <c r="G4" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" s="30"/>
+      <c r="K4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="L4" s="6">
+        <v>1</v>
+      </c>
+      <c r="M4" s="6">
+        <v>41</v>
+      </c>
+      <c r="N4" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
+      <c r="B5" s="46" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="45"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="6"/>
-      <c r="J5" s="3" t="s">
+      <c r="G5" s="31">
+        <v>244548</v>
+      </c>
+      <c r="H5" s="32"/>
+      <c r="K5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J6" s="3" t="s">
+      <c r="L5" s="6">
+        <v>45</v>
+      </c>
+      <c r="M5" s="6">
+        <v>72</v>
+      </c>
+      <c r="N5" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="K6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-    </row>
-    <row r="7" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="33" t="s">
+      <c r="L6" s="6">
+        <v>99</v>
+      </c>
+      <c r="M6" s="6">
+        <v>219</v>
+      </c>
+      <c r="N6" s="6">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A7" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="33" t="s">
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="33" t="s">
+      <c r="F7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="34" t="s">
+      <c r="G7" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="H7" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A8" s="33"/>
-      <c r="B8" s="8" t="s">
+      <c r="L7" s="6">
+        <v>100</v>
+      </c>
+      <c r="M7" s="6">
+        <v>220</v>
+      </c>
+      <c r="N7" s="6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A8" s="39"/>
+      <c r="B8" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="34"/>
-      <c r="J8" s="3" t="s">
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
+      <c r="K8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="L8" s="6">
+        <v>101</v>
+      </c>
+      <c r="M8" s="6">
+        <v>221</v>
+      </c>
+      <c r="N8" s="6">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B9" s="17">
+        <v>45</v>
+      </c>
+      <c r="C9" s="17">
+        <v>72</v>
+      </c>
+      <c r="D9" s="17">
+        <v>15</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B10" s="18">
+        <v>-1</v>
+      </c>
+      <c r="C10" s="43">
+        <v>72</v>
+      </c>
+      <c r="D10" s="43">
+        <v>15</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" s="26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="J11" s="2"/>
+      <c r="B11" s="18">
+        <v>0</v>
+      </c>
+      <c r="C11" s="43">
+        <v>72</v>
+      </c>
+      <c r="D11" s="43">
+        <v>15</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="27"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A12" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="J12" s="2"/>
+      <c r="B12" s="18">
+        <v>1</v>
+      </c>
+      <c r="C12" s="43">
+        <v>72</v>
+      </c>
+      <c r="D12" s="43">
+        <v>15</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" s="27"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A13" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="J13" s="2"/>
+      <c r="B13" s="18">
+        <v>99</v>
+      </c>
+      <c r="C13" s="43">
+        <v>72</v>
+      </c>
+      <c r="D13" s="43">
+        <v>15</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" s="27"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N13" s="2"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A14" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="J14" s="2"/>
+      <c r="B14" s="18">
+        <v>100</v>
+      </c>
+      <c r="C14" s="43">
+        <v>72</v>
+      </c>
+      <c r="D14" s="43">
+        <v>15</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="27"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
-    </row>
-    <row r="15" spans="1:13" s="36" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="35" t="s">
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A15" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="J15" s="37"/>
-      <c r="K15" s="37"/>
-      <c r="L15" s="37"/>
-      <c r="M15" s="37"/>
-    </row>
-    <row r="16" spans="1:13" s="36" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="35" t="s">
+      <c r="B15" s="18">
+        <v>101</v>
+      </c>
+      <c r="C15" s="43">
+        <v>72</v>
+      </c>
+      <c r="D15" s="43">
+        <v>15</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="28"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A16" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="J16" s="37"/>
-      <c r="K16" s="37"/>
-      <c r="L16" s="37"/>
-      <c r="M16" s="37"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B16" s="43">
+        <v>45</v>
+      </c>
+      <c r="C16" s="19">
+        <v>39</v>
+      </c>
+      <c r="D16" s="43">
+        <v>15</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A17" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="J17" s="2"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B17" s="43">
+        <v>45</v>
+      </c>
+      <c r="C17" s="19">
+        <v>40</v>
+      </c>
+      <c r="D17" s="43">
+        <v>15</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" s="27"/>
+      <c r="K17" s="2"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="J18" s="2"/>
+      <c r="B18" s="43">
+        <v>45</v>
+      </c>
+      <c r="C18" s="19">
+        <v>41</v>
+      </c>
+      <c r="D18" s="43">
+        <v>15</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H18" s="27"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N18" s="2"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A19" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B19" s="43">
+        <v>45</v>
+      </c>
+      <c r="C19" s="19">
+        <v>219</v>
+      </c>
+      <c r="D19" s="43">
+        <v>15</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H19" s="27"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A20" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A21" s="22" t="s">
+      <c r="B20" s="43">
+        <v>45</v>
+      </c>
+      <c r="C20" s="19">
+        <v>220</v>
+      </c>
+      <c r="D20" s="43">
+        <v>15</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H20" s="27"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A21" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="J21" s="2"/>
+      <c r="B21" s="43">
+        <v>45</v>
+      </c>
+      <c r="C21" s="19">
+        <v>221</v>
+      </c>
+      <c r="D21" s="43">
+        <v>15</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H21" s="28"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
-    </row>
-    <row r="22" spans="1:13" s="36" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="35" t="s">
+      <c r="N21" s="2"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A22" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="35"/>
-      <c r="J22" s="37"/>
-      <c r="K22" s="37"/>
-      <c r="L22" s="37"/>
-      <c r="M22" s="37"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="B22" s="43">
+        <v>45</v>
+      </c>
+      <c r="C22" s="43">
+        <v>72</v>
+      </c>
+      <c r="D22" s="24">
+        <v>-1</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H22" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A23" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="J23" s="2"/>
+      <c r="B23" s="43">
+        <v>45</v>
+      </c>
+      <c r="C23" s="43">
+        <v>72</v>
+      </c>
+      <c r="D23" s="24">
+        <v>0</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H23" s="27"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N23" s="2"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A24" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="J24" s="2"/>
+      <c r="B24" s="43">
+        <v>45</v>
+      </c>
+      <c r="C24" s="43">
+        <v>72</v>
+      </c>
+      <c r="D24" s="24">
+        <v>1</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" s="27"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N24" s="2"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A25" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="J25" s="2"/>
+      <c r="B25" s="43">
+        <v>45</v>
+      </c>
+      <c r="C25" s="43">
+        <v>72</v>
+      </c>
+      <c r="D25" s="24">
+        <v>29</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25" s="27"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.6">
       <c r="A26" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="J26" s="2"/>
+      <c r="B26" s="43">
+        <v>45</v>
+      </c>
+      <c r="C26" s="43">
+        <v>72</v>
+      </c>
+      <c r="D26" s="24">
+        <v>30</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H26" s="27"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
-    </row>
-    <row r="27" spans="1:13" s="36" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="35" t="s">
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.6">
+      <c r="A27" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
-      <c r="J27" s="37"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J28" s="2"/>
+      <c r="B27" s="43">
+        <v>45</v>
+      </c>
+      <c r="C27" s="43">
+        <v>72</v>
+      </c>
+      <c r="D27" s="24">
+        <v>31</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H27" s="28"/>
+      <c r="K27" s="2"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.6">
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="16">
+    <mergeCell ref="H10:H15"/>
+    <mergeCell ref="H16:H21"/>
+    <mergeCell ref="H22:H27"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
@@ -1776,21 +2555,32 @@
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F7:F8"/>
+    <mergeCell ref="H7:H8"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8068CBD9-38BE-794D-AE4F-17FC500CF117}">
-  <dimension ref="A2:K3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="27" x14ac:dyDescent="0.45"/>
+  <dimension ref="A2:K5"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="27" x14ac:dyDescent="0.6"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="2" width="10.875" style="1"/>
+    <col min="3" max="3" width="30.125" style="1" customWidth="1"/>
+    <col min="4" max="5" width="10.875" style="1"/>
+    <col min="6" max="6" width="16.125" style="1" customWidth="1"/>
+    <col min="7" max="10" width="10.875" style="1"/>
+    <col min="11" max="11" width="47" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="56" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="54" x14ac:dyDescent="0.6">
       <c r="A2" s="9" t="s">
         <v>23</v>
       </c>
@@ -1825,22 +2615,81 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A3" s="11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.6">
+      <c r="A3" s="48">
         <v>1</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
+      <c r="B3" s="48" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="47" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="49">
+        <v>244551</v>
+      </c>
+      <c r="E3" s="48" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="G3" s="48" t="s">
+        <v>88</v>
+      </c>
+      <c r="H3" s="48" t="s">
+        <v>89</v>
+      </c>
+      <c r="I3" s="48" t="s">
+        <v>90</v>
+      </c>
+      <c r="J3" s="48" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="50" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.6">
+      <c r="A4" s="48"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="47"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.6">
+      <c r="A5" s="48"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="47"/>
     </row>
   </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="K3:K5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="G3:G5"/>
+    <mergeCell ref="F3:F5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>